<commit_message>
slight update to naming
</commit_message>
<xml_diff>
--- a/Mouse brain RNAseq/sample_info_mouse_brain_rnaseq.xlsx
+++ b/Mouse brain RNAseq/sample_info_mouse_brain_rnaseq.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mchakra/Dropbox/Stanford/Research/Bhatt lab/Computation/BBB project/Paper code/Mouse brain RNAseq figures/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mchakra/Dropbox/Stanford/Research/Bhatt lab/Computation/BBB project/Paper code/Mouse brain RNAseq/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B524964-CF22-8140-853D-7DAEFCA79063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8BB9970-1E5B-E045-B29C-D6EAE9E2B235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="22640" windowHeight="17140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="45540" windowHeight="23180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
   <si>
     <t>Experiment</t>
   </si>
@@ -49,98 +49,110 @@
     <t>TMAO</t>
   </si>
   <si>
-    <t>TMAO_1</t>
-  </si>
-  <si>
-    <t>TMAO_2</t>
-  </si>
-  <si>
-    <t>TMAO_3</t>
-  </si>
-  <si>
-    <t>TMAO_4</t>
-  </si>
-  <si>
     <t>Saline</t>
-  </si>
-  <si>
-    <t>S_1</t>
-  </si>
-  <si>
-    <t>S_2</t>
-  </si>
-  <si>
-    <t>S_3</t>
-  </si>
-  <si>
-    <t>S_4</t>
   </si>
   <si>
     <t>GDCA</t>
   </si>
   <si>
-    <t>GDCA_1</t>
-  </si>
-  <si>
-    <t>GDCA_2</t>
-  </si>
-  <si>
-    <t>GDCA_3</t>
-  </si>
-  <si>
-    <t>GDCA_4</t>
-  </si>
-  <si>
     <t>PA</t>
-  </si>
-  <si>
-    <t>PA_1</t>
-  </si>
-  <si>
-    <t>PA_2</t>
-  </si>
-  <si>
-    <t>PA_3</t>
-  </si>
-  <si>
-    <t>PA_4</t>
   </si>
   <si>
     <t>IAA</t>
   </si>
   <si>
-    <t>IAA_1</t>
-  </si>
-  <si>
-    <t>IAA_2</t>
-  </si>
-  <si>
-    <t>IAA_3</t>
-  </si>
-  <si>
-    <t>IAA_4</t>
-  </si>
-  <si>
     <t>Saline + DMSO</t>
   </si>
   <si>
-    <t>SD_1</t>
+    <t>Expt1_TMAO1</t>
   </si>
   <si>
-    <t>SD_2</t>
+    <t>Expt1_TMAO2</t>
   </si>
   <si>
-    <t>SD_3</t>
+    <t>Expt1_TMAO3</t>
   </si>
   <si>
-    <t>SD_4</t>
+    <t>Expt1_TMAO4</t>
+  </si>
+  <si>
+    <t>Expt1_S1</t>
+  </si>
+  <si>
+    <t>Expt1_S2</t>
+  </si>
+  <si>
+    <t>Expt1_S3</t>
+  </si>
+  <si>
+    <t>Expt1_S4</t>
+  </si>
+  <si>
+    <t>Expt2_GDCA1</t>
+  </si>
+  <si>
+    <t>Expt2_GDCA2</t>
+  </si>
+  <si>
+    <t>Expt2_GDCA3</t>
+  </si>
+  <si>
+    <t>Expt2_GDCA4</t>
+  </si>
+  <si>
+    <t>Expt2_S1</t>
+  </si>
+  <si>
+    <t>Expt2_S2</t>
+  </si>
+  <si>
+    <t>Expt2_S3</t>
+  </si>
+  <si>
+    <t>Expt2_S4</t>
+  </si>
+  <si>
+    <t>Expt2_PA1</t>
+  </si>
+  <si>
+    <t>Expt2_PA2</t>
+  </si>
+  <si>
+    <t>Expt2_PA3</t>
+  </si>
+  <si>
+    <t>Expt2_PA4</t>
+  </si>
+  <si>
+    <t>Expt2_IAA1</t>
+  </si>
+  <si>
+    <t>Expt2_IAA2</t>
+  </si>
+  <si>
+    <t>Expt2_IAA3</t>
+  </si>
+  <si>
+    <t>Expt2_IAA4</t>
+  </si>
+  <si>
+    <t>Expt2_SD1</t>
+  </si>
+  <si>
+    <t>Expt2_SD2</t>
+  </si>
+  <si>
+    <t>Expt2_SD3</t>
+  </si>
+  <si>
+    <t>Expt2_SD4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -166,6 +178,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -188,7 +207,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -196,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -214,6 +233,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -496,7 +519,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E2" s="4">
         <v>9.4</v>
@@ -538,7 +561,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E3" s="4">
         <v>9.3000000000000007</v>
@@ -580,7 +603,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E4" s="4">
         <v>9.5</v>
@@ -622,7 +645,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E5" s="4">
         <v>9.5</v>
@@ -661,10 +684,10 @@
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E6" s="4">
         <v>9.5</v>
@@ -703,10 +726,10 @@
         <v>7</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E7" s="4">
         <v>9</v>
@@ -745,10 +768,10 @@
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E8" s="4">
         <v>9.3000000000000007</v>
@@ -779,7 +802,7 @@
       <c r="Y8" s="3"/>
       <c r="Z8" s="3"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5">
         <v>1</v>
       </c>
@@ -787,10 +810,10 @@
         <v>7</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E9" s="6">
         <v>9.3000000000000007</v>
@@ -829,10 +852,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E10" s="4">
         <v>8.9</v>
@@ -871,10 +894,10 @@
         <v>1</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E11" s="4">
         <v>9</v>
@@ -913,10 +936,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E12" s="4">
         <v>9.1</v>
@@ -955,10 +978,10 @@
         <v>1</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E13" s="4">
         <v>8.8000000000000007</v>
@@ -997,10 +1020,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="E14" s="4">
         <v>8.8000000000000007</v>
@@ -1039,10 +1062,10 @@
         <v>1</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E15" s="4">
         <v>9</v>
@@ -1081,10 +1104,10 @@
         <v>1</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="E16" s="4">
         <v>9</v>
@@ -1123,10 +1146,10 @@
         <v>1</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="E17" s="4">
         <v>9.1</v>
@@ -1165,10 +1188,10 @@
         <v>2</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>24</v>
+      <c r="D18" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="E18" s="4">
         <v>8.9</v>
@@ -1207,10 +1230,10 @@
         <v>2</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>25</v>
+      <c r="D19" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="E19" s="4">
         <v>9.1</v>
@@ -1249,10 +1272,10 @@
         <v>2</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>26</v>
+      <c r="D20" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="E20" s="4">
         <v>9.1</v>
@@ -1291,10 +1314,10 @@
         <v>2</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>27</v>
+      <c r="D21" s="8" t="s">
+        <v>33</v>
       </c>
       <c r="E21" s="4">
         <v>9.1</v>
@@ -1333,10 +1356,10 @@
         <v>2</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>29</v>
+      <c r="D22" s="8" t="s">
+        <v>34</v>
       </c>
       <c r="E22" s="4">
         <v>8.9</v>
@@ -1375,10 +1398,10 @@
         <v>2</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>30</v>
+      <c r="D23" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="E23" s="4">
         <v>9.3000000000000007</v>
@@ -1417,10 +1440,10 @@
         <v>2</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>31</v>
+      <c r="D24" s="8" t="s">
+        <v>36</v>
       </c>
       <c r="E24" s="4">
         <v>8.9</v>
@@ -1459,10 +1482,10 @@
         <v>2</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>32</v>
+      <c r="D25" s="8" t="s">
+        <v>37</v>
       </c>
       <c r="E25" s="4">
         <v>8.9</v>
@@ -1501,10 +1524,10 @@
         <v>2</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>34</v>
+      <c r="D26" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="E26" s="4">
         <v>8.9</v>
@@ -1543,10 +1566,10 @@
         <v>2</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>35</v>
+      <c r="D27" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="E27" s="4">
         <v>9</v>
@@ -1585,10 +1608,10 @@
         <v>2</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>36</v>
+      <c r="D28" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="E28" s="4">
         <v>8.9</v>
@@ -1627,10 +1650,10 @@
         <v>2</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>37</v>
+      <c r="D29" s="8" t="s">
+        <v>41</v>
       </c>
       <c r="E29" s="4">
         <v>9</v>

</xml_diff>